<commit_message>
T02: gable courses run over the corners to the outer face (corners no longer trimmed flat at the eaves)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/T02/downloads/DG-T02 Turnkey BOQ.xlsx
+++ b/T02/downloads/DG-T02 Turnkey BOQ.xlsx
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>7.59</v>
+        <v>7.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>51.32</v>
+        <v>51.44</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>

</xml_diff>